<commit_message>
Animate every headshot into the MAG logo, and sync with the master sheet
Every signature now loads a crossfade GIF from images/gifs/ on jsDelivr
@v1.1.0: the photo fades into the MAG logo and back. make-gifs.py builds
them from images/headshots/ and keeps the source of each in
images/gifs/sources.json. A signature image that fails to load on a page
is swapped for the logo before it can be copied.

From the master sheet (Google, 2026-10-12):
- 15 SA signatures move to the office line, 044 382 0565
- Anthony Lightening is Growth Marketer; Marie Hentschel is now Marie
  Bredenkamp, Account Director; Gabriel Arias is Web Developer on
  +49 151 26044084
- New starters with the logo until their headshot arrives: Hanli Janse
  van Rensburg, Marku Boshoff, Martin Frank, Reece Hurley, Ruan Killian,
  Victor Helberg, Zia Peter
- Gerrie van Niekerk and Gigh Zack removed (duplicates of Gerhardus Van
  Niekerk and Guy Zack)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAG-signatures-master.xlsx
+++ b/MAG-signatures-master.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signatures" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Signatures" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -588,13 +588,17 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>aimee-3-400x400-circle-v1.png</t>
+          <t>Aimee_Henley.gif</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Althia Kapp</t>
@@ -632,7 +636,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>althia-3-400x400-circle-v2.png</t>
+          <t>Althia_Kapp.gif</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr"/>
@@ -676,13 +680,17 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>annemarie-luck-400x400transparent.png</t>
+          <t>Annemarie_Luck.gif</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Anri van Der Linde</t>
@@ -700,7 +708,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>074 265 7444</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -720,13 +728,17 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>anri-2-400x400-circle-v1.png</t>
+          <t>Anri_van_Der_Linde.gif</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Anthony Lightening</t>
@@ -734,7 +746,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Digital Marketing Intern</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -744,7 +756,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>073 871 0480</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -764,7 +776,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>anthony-4-400x400-circle-v1.png</t>
+          <t>Anthony_Lightening.gif</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr"/>
@@ -808,13 +820,17 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>ashleigh-3-400x400-circle-v1.png</t>
+          <t>Ashleigh_van_Loggerenberg.gif</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Candice Masson</t>
@@ -852,13 +868,17 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>candice-2-400x400-circle-v1.png</t>
+          <t>Candice_Masson.gif</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Carla Engelbrecht</t>
@@ -876,7 +896,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>084 729 3414</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -896,7 +916,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>carla-4-400x400-circle-v1.png</t>
+          <t>Carla_Engelbrecht.gif</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr"/>
@@ -936,7 +956,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>elizabeth-danjean-400x400transparent.png</t>
+          <t>Elizabeth_Danjean.gif</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -946,7 +966,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Elizna Steyn</t>
@@ -984,7 +1008,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>elizna-4-400x400-circle-v1.png</t>
+          <t>Elizna_Steyn.gif</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
@@ -1028,13 +1052,17 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>elran-meiring-400x400transparent.png</t>
+          <t>Elran_Meiring.gif</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Etienne Bruwer</t>
@@ -1072,7 +1100,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>etienne-bruwer-400x400transparent.png</t>
+          <t>Etienne_Bruwer.gif</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr"/>
@@ -1116,7 +1144,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>eugene-4-400x400-circle-v1.png</t>
+          <t>Eugene_Bredenkamp.gif</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
@@ -1160,7 +1188,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>fergus-david-hannah-400x400transparent.png</t>
+          <t>Fergus_David_Hannah.gif</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
@@ -1204,13 +1232,17 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>gabrielle-zondagh-400x400transparent.png</t>
+          <t>Gabrielle_Zondagh.gif</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Gemma Persello</t>
@@ -1228,7 +1260,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>078 774 8835</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1248,39 +1280,43 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>gemma-2-400x400-circle-v1.png</t>
+          <t>Gemma_Persello.gif</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr"/>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Gerhardus Van Niekerk</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>CFO - Junior Partner</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>gerrie@mag.cr</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>084 200 0823</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Gerhardus_Van_Niekerk.html</t>
         </is>
@@ -1290,133 +1326,129 @@
           <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>gerrie-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Gerrie van Niekerk - one of these pages should go</t>
-        </is>
-      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Gerhardus_Van_Niekerk.gif</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Gerrie van Niekerk</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Junior Partner &amp; CFO</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>gerrie@mag.cr</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>084 200 0823</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Gerrie_van_Niekerk.html</t>
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Greg Hall</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SEO/PPC Specialist</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>greg@mag.cr</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>082 798 2660</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Greg_Hall.html</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gerrie_van_Niekerk.html</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>gerrie-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Gerhardus Van Niekerk - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Greg_Hall.html</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Greg_Hall.gif</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr"/>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Gigh Zack</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Guy Zack</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Animation Lead</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Guy@mag.cr</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>078 686 9971</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Gigh_Zack.html</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Guy_Zack.html</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gigh_Zack.html</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>gigh-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Guy Zack - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Guy_Zack.gif</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Greg Hall</t>
+          <t>Hanli Janse van Rensburg</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>SEO/PPC Specialist</t>
+          <t>Office Administration &amp; PA</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>greg@mag.cr</t>
+          <t>hanli@mag.cr</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>082 798 2660</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1426,118 +1458,118 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Greg_Hall.html</t>
+          <t>Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Greg_Hall.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>greg-hall-400x400transparent.png</t>
+          <t>Hanli_Janse_van_Rensburg.gif</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr"/>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Guy Zack</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Animation Lead</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Guy@mag.cr</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>078 686 9971</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Guy_Zack.html</t>
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Jean-Paul Brouard</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Designer</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>jp@mag.cr</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>083 997 7987</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Jean-Paul_Brouard.html</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>gigh-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Gigh Zack - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jean-Paul_Brouard.html</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Jean-Paul_Brouard.gif</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Jean-Paul Brouard</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Designer</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>jp@mag.cr</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>083 997 7987</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Jean-Paul_Brouard.html</t>
+      <c r="A23" s="6" t="inlineStr"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Jess van Anraad</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Junior Designer</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Jess@mag.cr</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>066 054 6464</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Jess_van_Anraad.html</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jean-Paul_Brouard.html</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>jean-paul-brouard-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr"/>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_Anraad.html</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>Jess_van_Anraad.gif</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Same address and headshot as Jess van der Merwe - one of these pages should go</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr"/>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Jess van Anraad</t>
+          <t>Jess van der Merwe</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1562,93 +1594,93 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Jess_van_Anraad.html</t>
+          <t>Jess_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_Anraad.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>jess-4-400x400-circle-v1.png</t>
+          <t>Jess_van_der_Merwe.gif</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>Same address and headshot as Jess van der Merwe - one of these pages should go</t>
+          <t>Same address and headshot as Jess van Anraad - one of these pages should go</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr"/>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Jess van der Merwe</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Junior Designer</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Jess@mag.cr</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>066 054 6464</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Jess_van_der_Merwe.html</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Jomarie Voges</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Financial Controller</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>jomarie@mag.cr</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_der_Merwe.html</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>jess-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Jess van Anraad - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Jomarie_Voges.gif</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr"/>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jomarie Voges</t>
+          <t>Kayla Spinelli</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Office Administration/PA</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>jomarie@mag.cr</t>
+          <t>Kayla@mag.cr</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>082 269 7542</t>
+          <t>081 476 6721</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1658,17 +1690,17 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.html</t>
+          <t>Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>jomarie-6-400x400-circle-v1.png</t>
+          <t>Kayla_Spinelli.gif</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
@@ -1677,22 +1709,22 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Kayla Spinelli</t>
+          <t>Kendel Falkson</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Office Administration/PA</t>
+          <t>PR Agent</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Kayla@mag.cr</t>
+          <t>Kendel@mag.cr</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>081 476 6721</t>
+          <t>082 905 2656</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1702,41 +1734,45 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.html</t>
+          <t>Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>kayla-spinelli-400x400transparent.png</t>
+          <t>Kendel_Falkson.gif</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Kendel Falkson</t>
+          <t>Lani Bruwer</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>PR Agent</t>
+          <t>Web Developer &amp; Information Architect</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Kendel@mag.cr</t>
+          <t>lani@mag.cr</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>082 905 2656</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1746,41 +1782,45 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.html</t>
+          <t>Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>kendel-falkson-400x400transparent.png</t>
+          <t>Lani_Bruwer.gif</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Lani Bruwer</t>
+          <t>LeeAnn Visser</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Web Developer &amp; Information Architect</t>
+          <t>Video Producer</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>lani@mag.cr</t>
+          <t>lee@mag.cr</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>084 452 2304</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1790,41 +1830,45 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.html</t>
+          <t>LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>lani-bruwer-400x400transparent.png</t>
+          <t>LeeAnn_Visser.gif</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn Visser</t>
+          <t>Marie Bredenkamp</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Video Producer</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>lee@mag.cr</t>
+          <t>marie@mag.cr</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>078 675 6476</t>
+          <t>076 943 5538</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1834,41 +1878,45 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.html</t>
+          <t>Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>lee-3-400x400-circle-v1.png</t>
+          <t>Marie_Hentschel.gif</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Marie Hentschel</t>
+          <t>Marku Boshoff</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Senior Account Manager</t>
+          <t>Video Editor</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>marie@mag.cr</t>
+          <t>marku@mag.cr</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>076 943 5538</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1878,41 +1926,45 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.html</t>
+          <t>Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>marie-4-400x400-circle-v1.png</t>
+          <t>Marku_Boshoff.gif</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Micaela Cox</t>
+          <t>Martin Frank</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Motion Graphics Designer</t>
+          <t>Creative Director</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Micaela@mag.cr</t>
+          <t>martin@mag.cr</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>082 977 5880</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1922,17 +1974,17 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.html</t>
+          <t>Martin_Frank.html</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>micaela-cox-400x400transparent.png</t>
+          <t>Martin_Frank.gif</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
@@ -1941,22 +1993,22 @@
       <c r="A33" s="2" t="inlineStr"/>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Mihlali Vumazonke</t>
+          <t>Micaela Cox</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Social Media Manager</t>
+          <t>Motion Graphics Designer</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Mihlali@mag.cr</t>
+          <t>Micaela@mag.cr</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>067 252 7987</t>
+          <t>082 977 5880</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -1966,17 +2018,17 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Mihlali_Vumazonke.html</t>
+          <t>Micaela_Cox.html</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mihlali_Vumazonke.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>mihlali-2-400x400-circle-v1.png</t>
+          <t>Micaela_Cox.gif</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
@@ -1985,86 +2037,90 @@
       <c r="A34" s="2" t="inlineStr"/>
       <c r="B34" s="3" t="inlineStr">
         <is>
+          <t>Mihlali Vumazonke</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Social Media Manager</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Mihlali@mag.cr</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>067 252 7987</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Mihlali_Vumazonke.html</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Mihlali_Vumazonke.html</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Mihlali_Vumazonke.gif</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
           <t>Monique Myburgh</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Growth Marketer</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>monique@mag.cr</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>072 317 2005</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Monique_Myburgh.html</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>monique-3-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Nicelle Bresler</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Senior Copywriter &amp; Strategist</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Nicell@mag.cr</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>082 295 1396</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Nicelle_Bresler.html</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
-        </is>
-      </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>nicelle-bresler-400x400transparent.png</t>
+          <t>Monique_Myburgh.gif</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr"/>
@@ -2073,198 +2129,214 @@
       <c r="A36" s="2" t="inlineStr"/>
       <c r="B36" s="3" t="inlineStr">
         <is>
+          <t>Nicelle Bresler</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Senior Copywriter &amp; Strategist</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Nicell@mag.cr</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>082 295 1396</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Nicelle_Bresler.html</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Nicelle_Bresler.gif</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
           <t>Noël Scholtz</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Director of Video</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>noel@mag.cr</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>072 070 5996</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Noël_Scholtz.html</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>noel-2-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J36" s="5" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Noël_Scholtz.html</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Noel_Scholtz.gif</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Nuhaa Davis</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Copywriter</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Nuhaa@mag.cr</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>079 467 4386</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Nuhaa_Davis.html</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>nuhaa-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Nuhaa_Davis.gif</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Portia Matha</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Junior Web Developer</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>portia@mag.cr</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>064 999 3847</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Portia_Matha.html</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>portia-2-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J38" s="5" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Riana Wiechers</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Copywriter</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>riana@mag.cr</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>063 687 4517</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Riana_Wiechers.html</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riana_Wiechers.html</t>
-        </is>
-      </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>riana-wiechers-400x400transparent.png</t>
+          <t>Portia_Matha.gif</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Riëtte Bester</t>
+          <t>Reece Hurley</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Junior Designer Intern</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>riette@mag.cr</t>
+          <t>reece@mag.cr</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>082 058 3483</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2274,17 +2346,17 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Riëtte_Bester.html</t>
+          <t>Reece_Hurley.html</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>riette-4-400x400-circle-v1.png</t>
+          <t>Reece_Hurley.gif</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
@@ -2293,1078 +2365,1398 @@
       <c r="A41" s="2" t="inlineStr"/>
       <c r="B41" s="3" t="inlineStr">
         <is>
+          <t>Riana Wiechers</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Copywriter</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>riana@mag.cr</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>063 687 4517</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Riana_Wiechers.html</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Riana_Wiechers.html</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Riana_Wiechers.gif</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Riëtte Bester</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Copywriter</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>riette@mag.cr</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Riëtte_Bester.html</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Riette_Bester.gif</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Ruan Killian</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Senior Designer</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>ruan@mag.cr</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Ruan_Killian.html</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Ruan_Killian.gif</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
           <t>Simeon Bezuidenhout</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Head of Video</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>simeon@mag.cr</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>071 462 0366</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Simeon_Bezuidenhout.html</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
         </is>
       </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>simeon-2-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J41" s="5" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Simeon_Bezuidenhout.gif</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Tshituku Ndadza</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Social Media Manager</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>Tshituku@mag.cr</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>078 593 5815</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Tshituku_Ndadza.html</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Tshituku_Ndadza.html</t>
         </is>
       </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>tshituku-2-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Tshituku_Ndadza.gif</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Victor Helberg</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Growth Marketer</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>victor@mag.cr</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Victor_Helberg.html</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Victor_Helberg.gif</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Willem van der Merwe</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Content Creator</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Willem@mag.cr</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>082 799 5884</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Willem_van_der_Merwe.html</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>willem-4-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Willem_van_der_Merwe.gif</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Zia Peter</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Senior Designer</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>zia@mag.cr</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Zia_Peter.html</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Zia_Peter.gif</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Adrian Mass</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>adrian@mag.cr</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>9515519165</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Adrian_Mass.html</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
-        <is>
-          <t>adrian-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr"/>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Adrian_Mass.gif</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr"/>
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>Bernadette Marconi</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>Senior Designer</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>bernadette@mag.cr</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>440-523-9455</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>Bernadette_Marconi.html</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Marconi.html</t>
         </is>
       </c>
-      <c r="I45" s="7" t="inlineStr">
-        <is>
-          <t>bernadette-marconi-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>Bernadette_Marconi.gif</t>
+        </is>
+      </c>
+      <c r="J50" s="8" t="inlineStr">
         <is>
           <t>Same address and headshot as Bernadette Rose Marconi - one of these pages should go</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr"/>
-      <c r="B46" s="7" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>Bernadette Rose Marconi</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>Senior Designer</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>bernadette@mag.cr</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>440-523-9455</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G51" s="7" t="inlineStr">
         <is>
           <t>Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
-      <c r="I46" s="7" t="inlineStr">
-        <is>
-          <t>bernadette-marconi-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J46" s="8" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>Bernadette_Rose_Marconi.gif</t>
+        </is>
+      </c>
+      <c r="J51" s="8" t="inlineStr">
         <is>
           <t>Same address and headshot as Bernadette Marconi - one of these pages should go</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="3" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Brad Hendrickson</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Junior Partner &amp; CCO</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>brad@mag.cr</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>818-231-7580</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Brad_Hendrickson.html</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>brad-hendrickson400x400.png</t>
-        </is>
-      </c>
-      <c r="J47" s="5" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Brad_Hendrickson.gif</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Brett Lorenz</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Head of Video Production</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>brett@mag.cr</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>865-323-0916</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Brett_Lorenz.html</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
-        <is>
-          <t>brett-lorenz-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Brett_Lorenz.gif</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Brittany Carlson</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>Account Operations Manager</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Brittany@mag.cr</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>951-225-5607</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Brittany_Carlson.html</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
         </is>
       </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>brittany-carlson-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Brittany_Carlson.gif</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Dave Korinek</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>Founding Partner</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>dave@mag.cr</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>858-395-6726</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Dave_Korinek.html</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>dave-korinek-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Dave_Korinek.gif</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>David Carrillo</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Partner &amp; ECD</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>dc@mag.cr</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>858-334-9855</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>David_Carrillo.html</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>david-carillo-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>David_Carrillo.gif</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Eric Kroupa</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Head of Content Strategy &amp; ACD</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>eric@mag.cr</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>636-236-8584</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G57" s="3" t="inlineStr">
         <is>
           <t>Eric_Kroupa.html</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>eric-kroupa-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Eric_Kroupa.gif</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Gabriel Arias</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Junior Web Developer</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Web Developer</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>gabriel@mag.cr</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>+584242038467</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>+49 151 26044084</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Gabriel_Arias.html</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>gabriel-arias-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Gabriel_Arias.gif</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Jorge Ramirez</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Head of Web Development</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>jorge@mag.cr</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>+502 5874-8315</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Jorge_Ramirez.html</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>jorge-ramirez-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J54" s="5" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Jorge_Ramirez.gif</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Lauren Spinelli</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Account Director</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>lauren@mag.cr</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>951-775-2078</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Lauren_Spinelli.html</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>lauren-spinelli-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr"/>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Lauren_Spinelli.gif</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr"/>
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>Mani Salazar</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>Design Director</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>mani@mag.cr</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E61" s="7" t="inlineStr">
         <is>
           <t>858-610-5380</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G61" s="7" t="inlineStr">
         <is>
           <t>Mani_Salazar.html</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Mani_Salazar.html</t>
         </is>
       </c>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>manuel-salazar-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J56" s="8" t="inlineStr">
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>Mani_Salazar.gif</t>
+        </is>
+      </c>
+      <c r="J61" s="8" t="inlineStr">
         <is>
           <t>Same address and headshot as Manuel Salazar - one of these pages should go</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr"/>
-      <c r="B57" s="7" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>Manuel Salazar</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>Design Director</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>mani@mag.cr</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E62" s="7" t="inlineStr">
         <is>
           <t>858-610-5380</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>Manuel_Salazar.html</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
         </is>
       </c>
-      <c r="I57" s="7" t="inlineStr">
-        <is>
-          <t>manuel-salazar-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J57" s="8" t="inlineStr">
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>Manuel_Salazar.gif</t>
+        </is>
+      </c>
+      <c r="J62" s="8" t="inlineStr">
         <is>
           <t>Same address and headshot as Mani Salazar - one of these pages should go</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
-      <c r="B58" s="3" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>Matt Simpson</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>Partner &amp; CGO</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>matt@mag.cr</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>858-705-2490</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Matt_Simpson.html</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr">
+      <c r="H63" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>matt-simpson-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J58" s="5" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr"/>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Matt_Simpson.gif</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Mia Pitino</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>HR/Operations Manager</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>mia@mag.cr</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>858-395-7142</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Mia_Pitino.html</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
         </is>
       </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>mia-pitino-400x400transparent-new.png</t>
-        </is>
-      </c>
-      <c r="J59" s="5" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Mia_Pitino.gif</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>Noah Korinek</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>noah@mag.cr</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>951-553-5340</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Noah_Korinek.html</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr">
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>noah-korinek-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J60" s="5" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr"/>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Noah_Korinek.gif</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Owen Korinek</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Videographer/Editor</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>owen@mag.cr</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>9515955535</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Owen_Korinek.html</t>
         </is>
       </c>
-      <c r="H61" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
         </is>
       </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>owen-400x400-circle-v1.png</t>
-        </is>
-      </c>
-      <c r="J61" s="5" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Owen_Korinek.gif</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>Paul Venter</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>paul@mag.cr</t>
         </is>
       </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>858-999-7975</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G62" s="3" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>Paul_Venter.html</t>
         </is>
       </c>
-      <c r="H62" s="4" t="inlineStr">
+      <c r="H67" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Paul_Venter.html</t>
         </is>
       </c>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>paul-venter-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J62" s="5" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr"/>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Paul_Venter.gif</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Thomas Condry</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>thomas@mag.cr</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>909-210-7305</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>Thomas_Condry.html</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
         </is>
       </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>thomas-condry-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J63" s="5" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr"/>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Thomas_Condry.gif</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>Tommy Eggert</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>tommy@mag.cr</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>858-243-1246</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G69" s="3" t="inlineStr">
         <is>
           <t>Tommy_Eggert.html</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>https://magn3tic.github.io/mag-signatures/pages/Tommy_Eggert.html</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>thomas-eggert-400x400transparent.png</t>
-        </is>
-      </c>
-      <c r="J64" s="5" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Tommy_Eggert.gif</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J64"/>
+  <autoFilter ref="A1:J69"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
+    <dataValidation sqref="A2:A69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
       <formula1>"Keep,Remove"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3432,6 +3824,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3462,7 +3859,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Every person who currently has a signature page. 63 rows.</t>
+          <t>Every person who currently has a signature page. 68 rows.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the 14 signatures that are no longer on the master sheet
Bernadette Marconi and Mani Salazar were duplicates of Bernadette Rose
Marconi and Manuel Salazar. Aimee Henley, Annemarie Luck, Ashleigh van
Loggerenberg, Elizabeth Danjean, Eugene Bredenkamp, Greg Hall, Jean-Paul
Brouard, Jess van Anraad, Jess van der Merwe, Mihlali Vumazonke, Riana
Wiechers and Tshituku Ndadza have left. Their headshots stay in images/
for the emails they already sent; their GIFs were never in a signature
that went out, so those go.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAG-signatures-master.xlsx
+++ b/MAG-signatures-master.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -54,7 +54,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF232323"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFDF8EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +85,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -103,15 +98,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -482,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -550,25 +536,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Aimee Henley</t>
+          <t>Althia Kapp</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Office Administration &amp; PA</t>
+          <t>Senior Account Manager</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>aimee@mag.cr</t>
+          <t>althia@mag.cr</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>082 922 6904</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -578,17 +568,17 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Aimee_Henley.html</t>
+          <t>Althia_Kapp.html</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Aimee_Henley.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Althia_Kapp.html</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Aimee_Henley.gif</t>
+          <t>Althia_Kapp.gif</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr"/>
@@ -601,22 +591,22 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Althia Kapp</t>
+          <t>Anri van Der Linde</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Senior Account Manager</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>althia@mag.cr</t>
+          <t>anri@mag.cr</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>082 922 6904</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -626,41 +616,45 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Althia_Kapp.html</t>
+          <t>Anri_van_Der_Linde.html</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Althia_Kapp.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Anri_van_Der_Linde.html</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Althia_Kapp.gif</t>
+          <t>Anri_van_Der_Linde.gif</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Annemarie Luck</t>
+          <t>Anthony Lightening</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Head of Strategy</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>annemarie@mag.cr</t>
+          <t>anthony@mag.cr</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>084 999 5257</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -670,17 +664,17 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Annemarie_Luck.html</t>
+          <t>Anthony_Lightening.html</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Annemarie_Luck.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Anthony_Lightening.html</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Annemarie_Luck.gif</t>
+          <t>Anthony_Lightening.gif</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr"/>
@@ -693,22 +687,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Anri van Der Linde</t>
+          <t>Candice Masson</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Director of Growth</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>anri@mag.cr</t>
+          <t>candice@mag.cr</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>078 544 7782</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -718,17 +712,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Anri_van_Der_Linde.html</t>
+          <t>Candice_Masson.html</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Anri_van_Der_Linde.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Candice_Masson.html</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Anri_van_Der_Linde.gif</t>
+          <t>Candice_Masson.gif</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr"/>
@@ -741,17 +735,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Anthony Lightening</t>
+          <t>Carla Engelbrecht</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Junior Designer</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>anthony@mag.cr</t>
+          <t>carla@mag.cr</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -766,41 +760,45 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Anthony_Lightening.html</t>
+          <t>Carla_Engelbrecht.html</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Anthony_Lightening.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Carla_Engelbrecht.html</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Anthony_Lightening.gif</t>
+          <t>Carla_Engelbrecht.gif</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ashleigh van Loggerenberg</t>
+          <t>Elizna Steyn</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Junior Copywriter</t>
+          <t>Account Manager</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Ashleigh@mag.cr</t>
+          <t>Elizna@mag.cr</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>064 365 4467</t>
+          <t>083 950 5998</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -810,17 +808,17 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Ashleigh_van_Loggerenberg.html</t>
+          <t>Elizna_Steyn.html</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Ashleigh_van_Loggerenberg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Elizna_Steyn.html</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Ashleigh_van_Loggerenberg.gif</t>
+          <t>Elizna_Steyn.gif</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr"/>
@@ -833,22 +831,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Candice Masson</t>
+          <t>Elran Meiring</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Director of Growth</t>
+          <t>Director of Paid Media</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>candice@mag.cr</t>
+          <t>Elran@mag.cr</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>078 544 7782</t>
+          <t>071 494 5189</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -858,17 +856,17 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Candice_Masson.html</t>
+          <t>Elran_Meiring.html</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Candice_Masson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Elran_Meiring.html</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Candice_Masson.gif</t>
+          <t>Elran_Meiring.gif</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr"/>
@@ -881,22 +879,22 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Carla Engelbrecht</t>
+          <t>Etienne Bruwer</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Junior Designer</t>
+          <t>Founding Partner &amp; CEO</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>carla@mag.cr</t>
+          <t>etienne@mag.cr</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>082 305 8213</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -906,64 +904,68 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Carla_Engelbrecht.html</t>
+          <t>Etienne_Bruwer.html</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Carla_Engelbrecht.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Etienne_Bruwer.html</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Carla_Engelbrecht.gif</t>
+          <t>Etienne_Bruwer.gif</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Elizabeth Danjean</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Jr Researcher and Brand Strategist</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>elizabeth@mag.cr</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Elizabeth_Danjean.html</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Fergus David Hannah</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Videographer/Editor</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>fergus@mag.cr</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>082 411 3920</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Fergus_David_Hannah.html</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Elizabeth_Danjean.html</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>Elizabeth_Danjean.gif</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>Phone row links to an empty tel: - fill it in or drop the row</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Fergus_David_Hannah.html</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Fergus_David_Hannah.gif</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -973,22 +975,22 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Elizna Steyn</t>
+          <t>Gabrielle Zondagh</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Account Manager</t>
+          <t>Account Coordinator</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Elizna@mag.cr</t>
+          <t>Gabrielle@mag.cr</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>083 950 5998</t>
+          <t>072 225 4850</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -998,41 +1000,45 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Elizna_Steyn.html</t>
+          <t>Gabrielle_Zondagh.html</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Elizna_Steyn.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gabrielle_Zondagh.html</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Elizna_Steyn.gif</t>
+          <t>Gabrielle_Zondagh.gif</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Elran Meiring</t>
+          <t>Gemma Persello</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Director of Paid Media</t>
+          <t>Senior Social Media Strategist</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Elran@mag.cr</t>
+          <t>gemma@mag.cr</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>071 494 5189</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1042,17 +1048,17 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Elran_Meiring.html</t>
+          <t>Gemma_Persello.html</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Elran_Meiring.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Elran_Meiring.gif</t>
+          <t>Gemma_Persello.gif</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr"/>
@@ -1065,22 +1071,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Etienne Bruwer</t>
+          <t>Gerhardus Van Niekerk</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Founding Partner &amp; CEO</t>
+          <t>CFO - Junior Partner</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>etienne@mag.cr</t>
+          <t>gerrie@mag.cr</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>082 305 8213</t>
+          <t>084 200 0823</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1090,41 +1096,45 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Etienne_Bruwer.html</t>
+          <t>Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Etienne_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Etienne_Bruwer.gif</t>
+          <t>Gerhardus_Van_Niekerk.gif</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Eugene Bredenkamp</t>
+          <t>Guy Zack</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Studio Director</t>
+          <t>Animation Lead</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>eugene@mag.cr</t>
+          <t>Guy@mag.cr</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>079 060 7844</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1134,41 +1144,45 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Eugene_Bredenkamp.html</t>
+          <t>Guy_Zack.html</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Eugene_Bredenkamp.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Eugene_Bredenkamp.gif</t>
+          <t>Guy_Zack.gif</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Fergus David Hannah</t>
+          <t>Hanli Janse van Rensburg</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Videographer/Editor</t>
+          <t>Office Administration &amp; PA</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>fergus@mag.cr</t>
+          <t>hanli@mag.cr</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>082 411 3920</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1178,41 +1192,45 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Fergus_David_Hannah.html</t>
+          <t>Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Fergus_David_Hannah.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Fergus_David_Hannah.gif</t>
+          <t>Hanli_Janse_van_Rensburg.gif</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle Zondagh</t>
+          <t>Jomarie Voges</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Account Coordinator</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle@mag.cr</t>
+          <t>jomarie@mag.cr</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>072 225 4850</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1222,17 +1240,17 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.html</t>
+          <t>Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabrielle_Zondagh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.gif</t>
+          <t>Jomarie_Voges.gif</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
@@ -1245,22 +1263,22 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Gemma Persello</t>
+          <t>Kayla Spinelli</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Senior Social Media Strategist</t>
+          <t>Office Administration/PA</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>gemma@mag.cr</t>
+          <t>Kayla@mag.cr</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>081 476 6721</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1270,17 +1288,17 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.html</t>
+          <t>Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.gif</t>
+          <t>Kayla_Spinelli.gif</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
@@ -1293,22 +1311,22 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus Van Niekerk</t>
+          <t>Kendel Falkson</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>CFO - Junior Partner</t>
+          <t>PR Agent</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>gerrie@mag.cr</t>
+          <t>Kendel@mag.cr</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>084 200 0823</t>
+          <t>082 905 2656</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1318,41 +1336,45 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.html</t>
+          <t>Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.gif</t>
+          <t>Kendel_Falkson.gif</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Greg Hall</t>
+          <t>Lani Bruwer</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>SEO/PPC Specialist</t>
+          <t>Web Developer &amp; Information Architect</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>greg@mag.cr</t>
+          <t>lani@mag.cr</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>082 798 2660</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1362,17 +1384,17 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Greg_Hall.html</t>
+          <t>Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Greg_Hall.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Greg_Hall.gif</t>
+          <t>Lani_Bruwer.gif</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr"/>
@@ -1385,17 +1407,17 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Guy Zack</t>
+          <t>LeeAnn Visser</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Animation Lead</t>
+          <t>Video Producer</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Guy@mag.cr</t>
+          <t>lee@mag.cr</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1410,17 +1432,17 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.html</t>
+          <t>LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.gif</t>
+          <t>LeeAnn_Visser.gif</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
@@ -1433,68 +1455,72 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Hanli Janse van Rensburg</t>
+          <t>Marie Bredenkamp</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Office Administration &amp; PA</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>hanli@mag.cr</t>
+          <t>marie@mag.cr</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>076 943 5538</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Marie_Hentschel.html</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Marie_Hentschel.gif</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Marku Boshoff</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Video Editor</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>marku@mag.cr</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
           <t>044 382 0565</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Hanli_Janse_van_Rensburg.html</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Hanli_Janse_van_Rensburg.gif</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Jean-Paul Brouard</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Designer</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>jp@mag.cr</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>083 997 7987</t>
-        </is>
-      </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
           <t>South Africa</t>
@@ -1502,116 +1528,116 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Jean-Paul_Brouard.html</t>
+          <t>Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jean-Paul_Brouard.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Jean-Paul_Brouard.gif</t>
+          <t>Marku_Boshoff.gif</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr"/>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Jess van Anraad</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Junior Designer</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Jess@mag.cr</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>066 054 6464</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Jess_van_Anraad.html</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Martin Frank</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Creative Director</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>martin@mag.cr</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>044 382 0565</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Martin_Frank.html</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_Anraad.html</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Jess_van_Anraad.gif</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Jess van der Merwe - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Martin_Frank.gif</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr"/>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Jess van der Merwe</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Junior Designer</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Jess@mag.cr</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>066 054 6464</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Jess_van_der_Merwe.html</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Micaela Cox</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Motion Graphics Designer</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Micaela@mag.cr</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>082 977 5880</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Micaela_Cox.html</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jess_van_der_Merwe.html</t>
-        </is>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>Jess_van_der_Merwe.gif</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Jess van Anraad - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Micaela_Cox.gif</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1621,17 +1647,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Jomarie Voges</t>
+          <t>Monique Myburgh</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>jomarie@mag.cr</t>
+          <t>monique@mag.cr</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1646,41 +1672,45 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.html</t>
+          <t>Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.gif</t>
+          <t>Monique_Myburgh.gif</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Kayla Spinelli</t>
+          <t>Nicelle Bresler</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Office Administration/PA</t>
+          <t>Senior Copywriter &amp; Strategist</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Kayla@mag.cr</t>
+          <t>Nicell@mag.cr</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>081 476 6721</t>
+          <t>082 295 1396</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1690,41 +1720,45 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.html</t>
+          <t>Nicelle_Bresler.html</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.gif</t>
+          <t>Nicelle_Bresler.gif</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Kendel Falkson</t>
+          <t>Noël Scholtz</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>PR Agent</t>
+          <t>Director of Video</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Kendel@mag.cr</t>
+          <t>noel@mag.cr</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>082 905 2656</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1734,17 +1768,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.html</t>
+          <t>Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.gif</t>
+          <t>Noel_Scholtz.gif</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr"/>
@@ -1757,17 +1791,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Lani Bruwer</t>
+          <t>Nuhaa Davis</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Web Developer &amp; Information Architect</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>lani@mag.cr</t>
+          <t>Nuhaa@mag.cr</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1782,17 +1816,17 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.html</t>
+          <t>Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.gif</t>
+          <t>Nuhaa_Davis.gif</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
@@ -1805,17 +1839,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn Visser</t>
+          <t>Portia Matha</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Video Producer</t>
+          <t>Junior Web Developer</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>lee@mag.cr</t>
+          <t>portia@mag.cr</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1830,17 +1864,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.html</t>
+          <t>Portia_Matha.html</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.gif</t>
+          <t>Portia_Matha.gif</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
@@ -1853,22 +1887,22 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Marie Bredenkamp</t>
+          <t>Reece Hurley</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Account Director</t>
+          <t>Junior Designer Intern</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>marie@mag.cr</t>
+          <t>reece@mag.cr</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>076 943 5538</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1878,17 +1912,17 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.html</t>
+          <t>Reece_Hurley.html</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.gif</t>
+          <t>Reece_Hurley.gif</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
@@ -1901,17 +1935,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Marku Boshoff</t>
+          <t>Riëtte Bester</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Video Editor</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>marku@mag.cr</t>
+          <t>riette@mag.cr</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1926,17 +1960,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.html</t>
+          <t>Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.gif</t>
+          <t>Riette_Bester.gif</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
@@ -1949,17 +1983,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Martin Frank</t>
+          <t>Ruan Killian</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Creative Director</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>martin@mag.cr</t>
+          <t>ruan@mag.cr</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1974,41 +2008,45 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.html</t>
+          <t>Ruan_Killian.html</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.gif</t>
+          <t>Ruan_Killian.gif</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Micaela Cox</t>
+          <t>Simeon Bezuidenhout</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Motion Graphics Designer</t>
+          <t>Head of Video</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Micaela@mag.cr</t>
+          <t>simeon@mag.cr</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>082 977 5880</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2018,41 +2056,45 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.html</t>
+          <t>Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.gif</t>
+          <t>Simeon_Bezuidenhout.gif</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Mihlali Vumazonke</t>
+          <t>Victor Helberg</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Social Media Manager</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Mihlali@mag.cr</t>
+          <t>victor@mag.cr</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>067 252 7987</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2062,17 +2104,17 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Mihlali_Vumazonke.html</t>
+          <t>Victor_Helberg.html</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mihlali_Vumazonke.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Mihlali_Vumazonke.gif</t>
+          <t>Victor_Helberg.gif</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr"/>
@@ -2085,17 +2127,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Monique Myburgh</t>
+          <t>Willem van der Merwe</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>monique@mag.cr</t>
+          <t>Willem@mag.cr</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2110,41 +2152,45 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.html</t>
+          <t>Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.gif</t>
+          <t>Willem_van_der_Merwe.gif</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Nicelle Bresler</t>
+          <t>Zia Peter</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Senior Copywriter &amp; Strategist</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Nicell@mag.cr</t>
+          <t>zia@mag.cr</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>082 295 1396</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2154,17 +2200,17 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.html</t>
+          <t>Zia_Peter.html</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.gif</t>
+          <t>Zia_Peter.gif</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
@@ -2177,42 +2223,42 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Noël Scholtz</t>
+          <t>Adrian Mass</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Director of Video</t>
+          <t>Account Manager</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>noel@mag.cr</t>
+          <t>adrian@mag.cr</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>9515519165</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Noël_Scholtz.html</t>
+          <t>Adrian_Mass.html</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Noel_Scholtz.gif</t>
+          <t>Adrian_Mass.gif</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr"/>
@@ -2225,42 +2271,42 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa Davis</t>
+          <t>Bernadette Rose Marconi</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa@mag.cr</t>
+          <t>bernadette@mag.cr</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>440-523-9455</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.html</t>
+          <t>Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.gif</t>
+          <t>Bernadette_Rose_Marconi.gif</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
@@ -2273,42 +2319,42 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Portia Matha</t>
+          <t>Brad Hendrickson</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Junior Web Developer</t>
+          <t>Junior Partner &amp; CCO</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>portia@mag.cr</t>
+          <t>brad@mag.cr</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>818-231-7580</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.html</t>
+          <t>Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.gif</t>
+          <t>Brad_Hendrickson.gif</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
@@ -2321,86 +2367,90 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Reece Hurley</t>
+          <t>Brett Lorenz</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Junior Designer Intern</t>
+          <t>Head of Video Production</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>reece@mag.cr</t>
+          <t>brett@mag.cr</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>865-323-0916</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.html</t>
+          <t>Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.gif</t>
+          <t>Brett_Lorenz.gif</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Riana Wiechers</t>
+          <t>Brittany Carlson</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Account Operations Manager</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>riana@mag.cr</t>
+          <t>Brittany@mag.cr</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>063 687 4517</t>
+          <t>951-225-5607</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Riana_Wiechers.html</t>
+          <t>Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riana_Wiechers.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Riana_Wiechers.gif</t>
+          <t>Brittany_Carlson.gif</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr"/>
@@ -2413,42 +2463,42 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Riëtte Bester</t>
+          <t>Dave Korinek</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Founding Partner</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>riette@mag.cr</t>
+          <t>dave@mag.cr</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>858-395-6726</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Riëtte_Bester.html</t>
+          <t>Dave_Korinek.html</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Riette_Bester.gif</t>
+          <t>Dave_Korinek.gif</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr"/>
@@ -2461,42 +2511,42 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Ruan Killian</t>
+          <t>David Carrillo</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Partner &amp; ECD</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ruan@mag.cr</t>
+          <t>dc@mag.cr</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>858-334-9855</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.html</t>
+          <t>David_Carrillo.html</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.gif</t>
+          <t>David_Carrillo.gif</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
@@ -2509,86 +2559,90 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Simeon Bezuidenhout</t>
+          <t>Eric Kroupa</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Head of Video</t>
+          <t>Head of Content Strategy &amp; ACD</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>simeon@mag.cr</t>
+          <t>eric@mag.cr</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>636-236-8584</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.html</t>
+          <t>Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.gif</t>
+          <t>Eric_Kroupa.gif</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Tshituku Ndadza</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Social Media Manager</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Tshituku@mag.cr</t>
+          <t>gabriel@mag.cr</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>078 593 5815</t>
+          <t>+49 151 26044084</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Tshituku_Ndadza.html</t>
+          <t>Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Tshituku_Ndadza.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Tshituku_Ndadza.gif</t>
+          <t>Gabriel_Arias.gif</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr"/>
@@ -2601,42 +2655,42 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Victor Helberg</t>
+          <t>Jorge Ramirez</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Head of Web Development</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>victor@mag.cr</t>
+          <t>jorge@mag.cr</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>+502 5874-8315</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.html</t>
+          <t>Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.gif</t>
+          <t>Jorge_Ramirez.gif</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
@@ -2649,42 +2703,42 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Willem van der Merwe</t>
+          <t>Lauren Spinelli</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Content Creator</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Willem@mag.cr</t>
+          <t>lauren@mag.cr</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>951-775-2078</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.html</t>
+          <t>Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.gif</t>
+          <t>Lauren_Spinelli.gif</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr"/>
@@ -2697,42 +2751,42 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Zia Peter</t>
+          <t>Manuel Salazar</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Design Director</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>zia@mag.cr</t>
+          <t>mani@mag.cr</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>858-610-5380</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.html</t>
+          <t>Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.gif</t>
+          <t>Manuel_Salazar.gif</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr"/>
@@ -2745,22 +2799,22 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Adrian Mass</t>
+          <t>Matt Simpson</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Account Manager</t>
+          <t>Partner &amp; CGO</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>adrian@mag.cr</t>
+          <t>matt@mag.cr</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>9515519165</t>
+          <t>858-705-2490</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2770,120 +2824,116 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.html</t>
+          <t>Matt_Simpson.html</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.gif</t>
+          <t>Matt_Simpson.gif</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr"/>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette Marconi</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>Senior Designer</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>bernadette@mag.cr</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>440-523-9455</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Mia Pitino</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>HR/Operations Manager</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>mia@mag.cr</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>858-395-7142</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette_Marconi.html</t>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Mia_Pitino.html</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Marconi.html</t>
-        </is>
-      </c>
-      <c r="I50" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette_Marconi.gif</t>
-        </is>
-      </c>
-      <c r="J50" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Bernadette Rose Marconi - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Mia_Pitino.gif</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette Rose Marconi</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Senior Designer</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>bernadette@mag.cr</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>440-523-9455</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Noah Korinek</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Designer</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>noah@mag.cr</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>951-553-5340</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette_Rose_Marconi.html</t>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Noah_Korinek.html</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
-        </is>
-      </c>
-      <c r="I51" s="7" t="inlineStr">
-        <is>
-          <t>Bernadette_Rose_Marconi.gif</t>
-        </is>
-      </c>
-      <c r="J51" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Bernadette Marconi - one of these pages should go</t>
-        </is>
-      </c>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Noah_Korinek.gif</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2893,22 +2943,22 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Brad Hendrickson</t>
+          <t>Owen Korinek</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Junior Partner &amp; CCO</t>
+          <t>Videographer/Editor</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>brad@mag.cr</t>
+          <t>owen@mag.cr</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>818-231-7580</t>
+          <t>9515955535</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2918,17 +2968,17 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.html</t>
+          <t>Owen_Korinek.html</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.gif</t>
+          <t>Owen_Korinek.gif</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr"/>
@@ -2941,22 +2991,22 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Brett Lorenz</t>
+          <t>Paul Venter</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Head of Video Production</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>brett@mag.cr</t>
+          <t>paul@mag.cr</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>865-323-0916</t>
+          <t>858-999-7975</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -2966,17 +3016,17 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.html</t>
+          <t>Paul_Venter.html</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Paul_Venter.html</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.gif</t>
+          <t>Paul_Venter.gif</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr"/>
@@ -2989,22 +3039,22 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Brittany Carlson</t>
+          <t>Thomas Condry</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Account Operations Manager</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Brittany@mag.cr</t>
+          <t>thomas@mag.cr</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>951-225-5607</t>
+          <t>909-210-7305</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -3014,17 +3064,17 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.html</t>
+          <t>Thomas_Condry.html</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.gif</t>
+          <t>Thomas_Condry.gif</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr"/>
@@ -3037,22 +3087,22 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Dave Korinek</t>
+          <t>Tommy Eggert</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Founding Partner</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>dave@mag.cr</t>
+          <t>tommy@mag.cr</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>858-395-6726</t>
+          <t>858-243-1246</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3062,701 +3112,25 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.html</t>
+          <t>Tommy_Eggert.html</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Tommy_Eggert.html</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.gif</t>
+          <t>Tommy_Eggert.gif</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr"/>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>David Carrillo</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Partner &amp; ECD</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>dc@mag.cr</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>858-334-9855</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>David_Carrillo.html</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>David_Carrillo.gif</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>Eric Kroupa</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Head of Content Strategy &amp; ACD</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>eric@mag.cr</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>636-236-8584</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>Eric_Kroupa.html</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
-        </is>
-      </c>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>Eric_Kroupa.gif</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>Gabriel Arias</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Web Developer</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>gabriel@mag.cr</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>+49 151 26044084</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Gabriel_Arias.html</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>Gabriel_Arias.gif</t>
-        </is>
-      </c>
-      <c r="J58" s="5" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Jorge Ramirez</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Head of Web Development</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>jorge@mag.cr</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>+502 5874-8315</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Jorge_Ramirez.html</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>Jorge_Ramirez.gif</t>
-        </is>
-      </c>
-      <c r="J59" s="5" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>Lauren Spinelli</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Account Director</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>lauren@mag.cr</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>951-775-2078</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Lauren_Spinelli.html</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
-        </is>
-      </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>Lauren_Spinelli.gif</t>
-        </is>
-      </c>
-      <c r="J60" s="5" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr"/>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>Mani Salazar</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>Design Director</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>mani@mag.cr</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>858-610-5380</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G61" s="7" t="inlineStr">
-        <is>
-          <t>Mani_Salazar.html</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mani_Salazar.html</t>
-        </is>
-      </c>
-      <c r="I61" s="7" t="inlineStr">
-        <is>
-          <t>Mani_Salazar.gif</t>
-        </is>
-      </c>
-      <c r="J61" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Manuel Salazar - one of these pages should go</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Manuel Salazar</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>Design Director</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>mani@mag.cr</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="inlineStr">
-        <is>
-          <t>858-610-5380</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
-        <is>
-          <t>Manuel_Salazar.html</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
-        </is>
-      </c>
-      <c r="I62" s="7" t="inlineStr">
-        <is>
-          <t>Manuel_Salazar.gif</t>
-        </is>
-      </c>
-      <c r="J62" s="8" t="inlineStr">
-        <is>
-          <t>Same address and headshot as Mani Salazar - one of these pages should go</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>Matt Simpson</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>Partner &amp; CGO</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>matt@mag.cr</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>858-705-2490</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>Matt_Simpson.html</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>Matt_Simpson.gif</t>
-        </is>
-      </c>
-      <c r="J63" s="5" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Mia Pitino</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>HR/Operations Manager</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>mia@mag.cr</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>858-395-7142</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Mia_Pitino.html</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
-        </is>
-      </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>Mia_Pitino.gif</t>
-        </is>
-      </c>
-      <c r="J64" s="5" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>Noah Korinek</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Designer</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>noah@mag.cr</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>951-553-5340</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>Noah_Korinek.html</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
-        </is>
-      </c>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t>Noah_Korinek.gif</t>
-        </is>
-      </c>
-      <c r="J65" s="5" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>Owen Korinek</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Videographer/Editor</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>owen@mag.cr</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>9515955535</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Owen_Korinek.html</t>
-        </is>
-      </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>Owen_Korinek.gif</t>
-        </is>
-      </c>
-      <c r="J66" s="5" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>Paul Venter</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>paul@mag.cr</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>858-999-7975</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>Paul_Venter.html</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Paul_Venter.html</t>
-        </is>
-      </c>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t>Paul_Venter.gif</t>
-        </is>
-      </c>
-      <c r="J67" s="5" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>Thomas Condry</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Designer</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>thomas@mag.cr</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>909-210-7305</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>Thomas_Condry.html</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>Thomas_Condry.gif</t>
-        </is>
-      </c>
-      <c r="J68" s="5" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>Tommy Eggert</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>Producer</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>tommy@mag.cr</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>858-243-1246</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>Tommy_Eggert.html</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Tommy_Eggert.html</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>Tommy_Eggert.gif</t>
-        </is>
-      </c>
-      <c r="J69" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
+  <autoFilter ref="A1:J55"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
+    <dataValidation sqref="A2:A55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
       <formula1>"Keep,Remove"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3815,20 +3189,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3847,127 +3207,127 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>MAG email signatures - master list</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr"/>
+      <c r="A2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Every person who currently has a signature page. 68 rows.</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Every person who currently has a signature page. 54 rows.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr"/>
+      <c r="A4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Someone left the company</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Set their Status to Remove, save the file, and run:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">    python3 generator/remove.py</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>That deletes pages/&lt;their file&gt;.html and rebuilds index.html. Their headshot</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>is left in images/ on purpose - old emails already sent still load it.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr"/>
+      <c r="A10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Someone's details changed</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Editing this sheet does not change a signature. The signature markup lives in</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>the page itself. Change it there, or send the new details to whoever rebuilds.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr"/>
+      <c r="A14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>The highlighted rows</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Rows tinted cream have something in Notes worth resolving - a duplicate page,</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>or a phone row that links nowhere.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr"/>
+      <c r="A18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>This file is generated</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>python3 generator/build-master.py overwrites it. Statuses you have typed are</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>read first and carried over, so a rebuild does not lose your work.</t>
         </is>

</xml_diff>

<commit_message>
Sync with the master sheet: new roles and names, 2 joiners, 2 leavers
- Roles: Dave Korinek, Eric Kroupa, Matt Simpson, Thomas Condry
- Names: Bernadette Marconi, Mani Salazar (page URLs unchanged)
- New, with the logo until a headshot: Frederik Dippenaar, Jade Weir-Smith
- Removed: Paul Venter, Tommy Eggert (headshots kept for sent emails)
- Artwork tag bumped to v1.4.0 for the two new GIFs

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAG-signatures-master.xlsx
+++ b/MAG-signatures-master.xlsx
@@ -968,29 +968,25 @@
       <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle Zondagh</t>
+          <t>Frederik Dippenaar</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Account Coordinator</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle@mag.cr</t>
+          <t>frederik@mag.cr</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>072 225 4850</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1000,17 +996,17 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.html</t>
+          <t>Frederik_Dippenaar.html</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabrielle_Zondagh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Frederik_Dippenaar.html</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.gif</t>
+          <t>Frederik_Dippenaar.gif</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
@@ -1023,22 +1019,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Gemma Persello</t>
+          <t>Gabrielle Zondagh</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Senior Social Media Strategist</t>
+          <t>Account Coordinator</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>gemma@mag.cr</t>
+          <t>Gabrielle@mag.cr</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>072 225 4850</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1048,17 +1044,17 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.html</t>
+          <t>Gabrielle_Zondagh.html</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gabrielle_Zondagh.html</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.gif</t>
+          <t>Gabrielle_Zondagh.gif</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr"/>
@@ -1071,22 +1067,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus Van Niekerk</t>
+          <t>Gemma Persello</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>CFO - Junior Partner</t>
+          <t>Senior Social Media Strategist</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>gerrie@mag.cr</t>
+          <t>gemma@mag.cr</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>084 200 0823</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1096,17 +1092,17 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.html</t>
+          <t>Gemma_Persello.html</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.gif</t>
+          <t>Gemma_Persello.gif</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr"/>
@@ -1119,22 +1115,22 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Guy Zack</t>
+          <t>Gerhardus Van Niekerk</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Animation Lead</t>
+          <t>CFO - Junior Partner</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Guy@mag.cr</t>
+          <t>gerrie@mag.cr</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>084 200 0823</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1144,17 +1140,17 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.html</t>
+          <t>Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.gif</t>
+          <t>Gerhardus_Van_Niekerk.gif</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
@@ -1167,17 +1163,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Hanli Janse van Rensburg</t>
+          <t>Guy Zack</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Office Administration &amp; PA</t>
+          <t>Animation Lead</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>hanli@mag.cr</t>
+          <t>Guy@mag.cr</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1192,17 +1188,17 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Hanli_Janse_van_Rensburg.html</t>
+          <t>Guy_Zack.html</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hanli_Janse_van_Rensburg.gif</t>
+          <t>Guy_Zack.gif</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
@@ -1215,17 +1211,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Jomarie Voges</t>
+          <t>Hanli Janse van Rensburg</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Office Administration &amp; PA</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>jomarie@mag.cr</t>
+          <t>hanli@mag.cr</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1240,45 +1236,41 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.html</t>
+          <t>Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.gif</t>
+          <t>Hanli_Janse_van_Rensburg.gif</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Kayla Spinelli</t>
+          <t>Jade Weir-Smith</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Office Administration/PA</t>
+          <t>Junior Growth Marketer</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Kayla@mag.cr</t>
+          <t>jade@mag.cr</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>081 476 6721</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1288,17 +1280,17 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.html</t>
+          <t>Jade_Weir-Smith.html</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jade_Weir-Smith.html</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.gif</t>
+          <t>Jade_Weir-Smith.gif</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
@@ -1311,22 +1303,22 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Kendel Falkson</t>
+          <t>Jomarie Voges</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>PR Agent</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Kendel@mag.cr</t>
+          <t>jomarie@mag.cr</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>082 905 2656</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1336,17 +1328,17 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.html</t>
+          <t>Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.gif</t>
+          <t>Jomarie_Voges.gif</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr"/>
@@ -1359,22 +1351,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Lani Bruwer</t>
+          <t>Kayla Spinelli</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Web Developer &amp; Information Architect</t>
+          <t>Office Administration/PA</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>lani@mag.cr</t>
+          <t>Kayla@mag.cr</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>081 476 6721</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1384,17 +1376,17 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.html</t>
+          <t>Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.gif</t>
+          <t>Kayla_Spinelli.gif</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr"/>
@@ -1407,22 +1399,22 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn Visser</t>
+          <t>Kendel Falkson</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Video Producer</t>
+          <t>PR Agent</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>lee@mag.cr</t>
+          <t>Kendel@mag.cr</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>082 905 2656</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1432,17 +1424,17 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.html</t>
+          <t>Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.gif</t>
+          <t>Kendel_Falkson.gif</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
@@ -1455,22 +1447,22 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Marie Bredenkamp</t>
+          <t>Lani Bruwer</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Account Director</t>
+          <t>Web Developer &amp; Information Architect</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>marie@mag.cr</t>
+          <t>lani@mag.cr</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>076 943 5538</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1480,17 +1472,17 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.html</t>
+          <t>Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.gif</t>
+          <t>Lani_Bruwer.gif</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
@@ -1503,17 +1495,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Marku Boshoff</t>
+          <t>LeeAnn Visser</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Video Editor</t>
+          <t>Video Producer</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>marku@mag.cr</t>
+          <t>lee@mag.cr</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1528,17 +1520,17 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.html</t>
+          <t>LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.gif</t>
+          <t>LeeAnn_Visser.gif</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
@@ -1551,22 +1543,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Martin Frank</t>
+          <t>Marie Bredenkamp</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Creative Director</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>martin@mag.cr</t>
+          <t>marie@mag.cr</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>076 943 5538</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1576,17 +1568,17 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.html</t>
+          <t>Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.gif</t>
+          <t>Marie_Hentschel.gif</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr"/>
@@ -1599,22 +1591,22 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Micaela Cox</t>
+          <t>Marku Boshoff</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Motion Graphics Designer</t>
+          <t>Video Editor</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Micaela@mag.cr</t>
+          <t>marku@mag.cr</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>082 977 5880</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1624,17 +1616,17 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.html</t>
+          <t>Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.gif</t>
+          <t>Marku_Boshoff.gif</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
@@ -1647,17 +1639,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Monique Myburgh</t>
+          <t>Martin Frank</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Creative Director</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>monique@mag.cr</t>
+          <t>martin@mag.cr</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1672,17 +1664,17 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.html</t>
+          <t>Martin_Frank.html</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.gif</t>
+          <t>Martin_Frank.gif</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr"/>
@@ -1695,22 +1687,22 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Nicelle Bresler</t>
+          <t>Micaela Cox</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Senior Copywriter &amp; Strategist</t>
+          <t>Motion Graphics Designer</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Nicell@mag.cr</t>
+          <t>Micaela@mag.cr</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>082 295 1396</t>
+          <t>082 977 5880</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1720,17 +1712,17 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.html</t>
+          <t>Micaela_Cox.html</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.gif</t>
+          <t>Micaela_Cox.gif</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
@@ -1743,17 +1735,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Noël Scholtz</t>
+          <t>Monique Myburgh</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Director of Video</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>noel@mag.cr</t>
+          <t>monique@mag.cr</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1768,17 +1760,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Noël_Scholtz.html</t>
+          <t>Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Noel_Scholtz.gif</t>
+          <t>Monique_Myburgh.gif</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr"/>
@@ -1791,22 +1783,22 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa Davis</t>
+          <t>Nicelle Bresler</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Senior Copywriter &amp; Strategist</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa@mag.cr</t>
+          <t>Nicell@mag.cr</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>082 295 1396</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1816,17 +1808,17 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.html</t>
+          <t>Nicelle_Bresler.html</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.gif</t>
+          <t>Nicelle_Bresler.gif</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
@@ -1839,17 +1831,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Portia Matha</t>
+          <t>Noël Scholtz</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Junior Web Developer</t>
+          <t>Director of Video</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>portia@mag.cr</t>
+          <t>noel@mag.cr</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1864,17 +1856,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.html</t>
+          <t>Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.gif</t>
+          <t>Noel_Scholtz.gif</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
@@ -1887,17 +1879,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Reece Hurley</t>
+          <t>Nuhaa Davis</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Junior Designer Intern</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>reece@mag.cr</t>
+          <t>Nuhaa@mag.cr</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1912,17 +1904,17 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.html</t>
+          <t>Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.gif</t>
+          <t>Nuhaa_Davis.gif</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
@@ -1935,17 +1927,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Riëtte Bester</t>
+          <t>Portia Matha</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Junior Web Developer</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>riette@mag.cr</t>
+          <t>portia@mag.cr</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1960,17 +1952,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Riëtte_Bester.html</t>
+          <t>Portia_Matha.html</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Riette_Bester.gif</t>
+          <t>Portia_Matha.gif</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
@@ -1983,17 +1975,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Ruan Killian</t>
+          <t>Reece Hurley</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Junior Designer Intern</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>ruan@mag.cr</t>
+          <t>reece@mag.cr</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -2008,17 +2000,17 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.html</t>
+          <t>Reece_Hurley.html</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.gif</t>
+          <t>Reece_Hurley.gif</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
@@ -2031,17 +2023,17 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Simeon Bezuidenhout</t>
+          <t>Riëtte Bester</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Head of Video</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>simeon@mag.cr</t>
+          <t>riette@mag.cr</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -2056,17 +2048,17 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.html</t>
+          <t>Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.gif</t>
+          <t>Riette_Bester.gif</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
@@ -2079,17 +2071,17 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Victor Helberg</t>
+          <t>Ruan Killian</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>victor@mag.cr</t>
+          <t>ruan@mag.cr</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2104,17 +2096,17 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.html</t>
+          <t>Ruan_Killian.html</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.gif</t>
+          <t>Ruan_Killian.gif</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr"/>
@@ -2127,17 +2119,17 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Willem van der Merwe</t>
+          <t>Simeon Bezuidenhout</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Content Creator</t>
+          <t>Head of Video</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Willem@mag.cr</t>
+          <t>simeon@mag.cr</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2152,17 +2144,17 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.html</t>
+          <t>Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.gif</t>
+          <t>Simeon_Bezuidenhout.gif</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr"/>
@@ -2175,17 +2167,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Zia Peter</t>
+          <t>Victor Helberg</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>zia@mag.cr</t>
+          <t>victor@mag.cr</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2200,17 +2192,17 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.html</t>
+          <t>Victor_Helberg.html</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.gif</t>
+          <t>Victor_Helberg.gif</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
@@ -2223,42 +2215,42 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Adrian Mass</t>
+          <t>Willem van der Merwe</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Account Manager</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>adrian@mag.cr</t>
+          <t>Willem@mag.cr</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>9515519165</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.html</t>
+          <t>Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.gif</t>
+          <t>Willem_van_der_Merwe.gif</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr"/>
@@ -2271,7 +2263,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Bernadette Rose Marconi</t>
+          <t>Zia Peter</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2281,32 +2273,32 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>bernadette@mag.cr</t>
+          <t>zia@mag.cr</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>440-523-9455</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Bernadette_Rose_Marconi.html</t>
+          <t>Zia_Peter.html</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Bernadette_Rose_Marconi.gif</t>
+          <t>Zia_Peter.gif</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
@@ -2319,22 +2311,22 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Brad Hendrickson</t>
+          <t>Adrian Mass</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Junior Partner &amp; CCO</t>
+          <t>Account Manager</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>brad@mag.cr</t>
+          <t>adrian@mag.cr</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>818-231-7580</t>
+          <t>9515519165</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2344,17 +2336,17 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.html</t>
+          <t>Adrian_Mass.html</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.gif</t>
+          <t>Adrian_Mass.gif</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
@@ -2367,22 +2359,22 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Brett Lorenz</t>
+          <t>Bernadette Marconi</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Head of Video Production</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>brett@mag.cr</t>
+          <t>bernadette@mag.cr</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>865-323-0916</t>
+          <t>440-523-9455</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2392,17 +2384,17 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.html</t>
+          <t>Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.gif</t>
+          <t>Bernadette_Rose_Marconi.gif</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
@@ -2415,22 +2407,22 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Brittany Carlson</t>
+          <t>Brad Hendrickson</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Account Operations Manager</t>
+          <t>Junior Partner &amp; CCO</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Brittany@mag.cr</t>
+          <t>brad@mag.cr</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>951-225-5607</t>
+          <t>818-231-7580</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2440,17 +2432,17 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.html</t>
+          <t>Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.gif</t>
+          <t>Brad_Hendrickson.gif</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr"/>
@@ -2463,22 +2455,22 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Dave Korinek</t>
+          <t>Brett Lorenz</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Founding Partner</t>
+          <t>Head of Video Production</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>dave@mag.cr</t>
+          <t>brett@mag.cr</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>858-395-6726</t>
+          <t>865-323-0916</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2488,17 +2480,17 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.html</t>
+          <t>Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.gif</t>
+          <t>Brett_Lorenz.gif</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr"/>
@@ -2511,22 +2503,22 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>David Carrillo</t>
+          <t>Brittany Carlson</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Partner &amp; ECD</t>
+          <t>Account Operations Manager</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>dc@mag.cr</t>
+          <t>Brittany@mag.cr</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>858-334-9855</t>
+          <t>951-225-5607</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2536,17 +2528,17 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>David_Carrillo.html</t>
+          <t>Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>David_Carrillo.gif</t>
+          <t>Brittany_Carlson.gif</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
@@ -2559,22 +2551,22 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Eric Kroupa</t>
+          <t>Dave Korinek</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Head of Content Strategy &amp; ACD</t>
+          <t>Founder | Chief Brand Officer</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>eric@mag.cr</t>
+          <t>dave@mag.cr</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>636-236-8584</t>
+          <t>858-395-6726</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2584,17 +2576,17 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Eric_Kroupa.html</t>
+          <t>Dave_Korinek.html</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Eric_Kroupa.gif</t>
+          <t>Dave_Korinek.gif</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
@@ -2607,22 +2599,22 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>David Carrillo</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Web Developer</t>
+          <t>Partner &amp; ECD</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>gabriel@mag.cr</t>
+          <t>dc@mag.cr</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>+49 151 26044084</t>
+          <t>858-334-9855</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2632,17 +2624,17 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Gabriel_Arias.html</t>
+          <t>David_Carrillo.html</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Gabriel_Arias.gif</t>
+          <t>David_Carrillo.gif</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr"/>
@@ -2655,22 +2647,22 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Jorge Ramirez</t>
+          <t>Eric Kroupa</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Head of Web Development</t>
+          <t>Director of Creative Strategy</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>jorge@mag.cr</t>
+          <t>eric@mag.cr</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>+502 5874-8315</t>
+          <t>636-236-8584</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2680,17 +2672,17 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Jorge_Ramirez.html</t>
+          <t>Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Jorge_Ramirez.gif</t>
+          <t>Eric_Kroupa.gif</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
@@ -2703,22 +2695,22 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Lauren Spinelli</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Account Director</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>lauren@mag.cr</t>
+          <t>gabriel@mag.cr</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>951-775-2078</t>
+          <t>+49 151 26044084</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -2728,17 +2720,17 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Lauren_Spinelli.html</t>
+          <t>Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Lauren_Spinelli.gif</t>
+          <t>Gabriel_Arias.gif</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr"/>
@@ -2751,22 +2743,22 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Manuel Salazar</t>
+          <t>Jorge Ramirez</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Design Director</t>
+          <t>Head of Web Development</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>mani@mag.cr</t>
+          <t>jorge@mag.cr</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>858-610-5380</t>
+          <t>+502 5874-8315</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2776,17 +2768,17 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Manuel_Salazar.html</t>
+          <t>Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Manuel_Salazar.gif</t>
+          <t>Jorge_Ramirez.gif</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr"/>
@@ -2799,22 +2791,22 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Matt Simpson</t>
+          <t>Lauren Spinelli</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Partner &amp; CGO</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>matt@mag.cr</t>
+          <t>lauren@mag.cr</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>858-705-2490</t>
+          <t>951-775-2078</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2824,17 +2816,17 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Matt_Simpson.html</t>
+          <t>Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Matt_Simpson.gif</t>
+          <t>Lauren_Spinelli.gif</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
@@ -2847,22 +2839,22 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Mia Pitino</t>
+          <t>Mani Salazar</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>HR/Operations Manager</t>
+          <t>Design Director</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>mia@mag.cr</t>
+          <t>mani@mag.cr</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>858-395-7142</t>
+          <t>858-610-5380</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2872,17 +2864,17 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Mia_Pitino.html</t>
+          <t>Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Mia_Pitino.gif</t>
+          <t>Manuel_Salazar.gif</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr"/>
@@ -2895,22 +2887,22 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Noah Korinek</t>
+          <t>Matt Simpson</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Partner &amp; COO</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>noah@mag.cr</t>
+          <t>matt@mag.cr</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>951-553-5340</t>
+          <t>858-705-2490</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -2920,17 +2912,17 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Noah_Korinek.html</t>
+          <t>Matt_Simpson.html</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Noah_Korinek.gif</t>
+          <t>Matt_Simpson.gif</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr"/>
@@ -2943,22 +2935,22 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Owen Korinek</t>
+          <t>Mia Pitino</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Videographer/Editor</t>
+          <t>HR/Operations Manager</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>owen@mag.cr</t>
+          <t>mia@mag.cr</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>9515955535</t>
+          <t>858-395-7142</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2968,17 +2960,17 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Owen_Korinek.html</t>
+          <t>Mia_Pitino.html</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Owen_Korinek.gif</t>
+          <t>Mia_Pitino.gif</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr"/>
@@ -2991,22 +2983,22 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Paul Venter</t>
+          <t>Noah Korinek</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>paul@mag.cr</t>
+          <t>noah@mag.cr</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>858-999-7975</t>
+          <t>951-553-5340</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -3016,17 +3008,17 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Paul_Venter.html</t>
+          <t>Noah_Korinek.html</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Paul_Venter.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Paul_Venter.gif</t>
+          <t>Noah_Korinek.gif</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr"/>
@@ -3039,22 +3031,22 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Thomas Condry</t>
+          <t>Owen Korinek</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Designer</t>
+          <t>Videographer/Editor</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>thomas@mag.cr</t>
+          <t>owen@mag.cr</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>909-210-7305</t>
+          <t>9515955535</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -3064,17 +3056,17 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Thomas_Condry.html</t>
+          <t>Owen_Korinek.html</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Thomas_Condry.gif</t>
+          <t>Owen_Korinek.gif</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr"/>
@@ -3087,22 +3079,22 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Tommy Eggert</t>
+          <t>Thomas Condry</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Senior Digital and Motion Designer</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>tommy@mag.cr</t>
+          <t>thomas@mag.cr</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>858-243-1246</t>
+          <t>909-210-7305</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3112,17 +3104,17 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Tommy_Eggert.html</t>
+          <t>Thomas_Condry.html</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Tommy_Eggert.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Tommy_Eggert.gif</t>
+          <t>Thomas_Condry.gif</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Remove the 7 logo-only signatures that are not on the master sheet
Elran Meiring, Fergus David Hannah, Gabrielle Zondagh, Kayla Spinelli,
Kendel Falkson, Micaela Cox, Nicelle Bresler. Their GIFs stay in images/
so emails already sent keep loading.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAG-signatures-master.xlsx
+++ b/MAG-signatures-master.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signatures'!$A$1:$J$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -831,22 +831,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Elran Meiring</t>
+          <t>Etienne Bruwer</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Director of Paid Media</t>
+          <t>Founding Partner &amp; CEO</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Elran@mag.cr</t>
+          <t>etienne@mag.cr</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>071 494 5189</t>
+          <t>082 305 8213</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -856,45 +856,41 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Elran_Meiring.html</t>
+          <t>Etienne_Bruwer.html</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Elran_Meiring.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Etienne_Bruwer.html</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Elran_Meiring.gif</t>
+          <t>Etienne_Bruwer.gif</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Etienne Bruwer</t>
+          <t>Frederik Dippenaar</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Founding Partner &amp; CEO</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>etienne@mag.cr</t>
+          <t>frederik@mag.cr</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>082 305 8213</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -904,17 +900,17 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Etienne_Bruwer.html</t>
+          <t>Frederik_Dippenaar.html</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Etienne_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Frederik_Dippenaar.html</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Etienne_Bruwer.gif</t>
+          <t>Frederik_Dippenaar.gif</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr"/>
@@ -927,22 +923,22 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Fergus David Hannah</t>
+          <t>Gemma Persello</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Videographer/Editor</t>
+          <t>Senior Social Media Strategist</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>fergus@mag.cr</t>
+          <t>gemma@mag.cr</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>082 411 3920</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -952,41 +948,45 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Fergus_David_Hannah.html</t>
+          <t>Gemma_Persello.html</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Fergus_David_Hannah.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Fergus_David_Hannah.gif</t>
+          <t>Gemma_Persello.gif</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Frederik Dippenaar</t>
+          <t>Gerhardus Van Niekerk</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Content Creator</t>
+          <t>CFO - Junior Partner</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>frederik@mag.cr</t>
+          <t>gerrie@mag.cr</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>084 200 0823</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -996,17 +996,17 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Frederik_Dippenaar.html</t>
+          <t>Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Frederik_Dippenaar.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Frederik_Dippenaar.gif</t>
+          <t>Gerhardus_Van_Niekerk.gif</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr"/>
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle Zondagh</t>
+          <t>Guy Zack</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Account Coordinator</t>
+          <t>Animation Lead</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle@mag.cr</t>
+          <t>Guy@mag.cr</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>072 225 4850</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1044,17 +1044,17 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.html</t>
+          <t>Guy_Zack.html</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabrielle_Zondagh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Gabrielle_Zondagh.gif</t>
+          <t>Guy_Zack.gif</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr"/>
@@ -1067,17 +1067,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Gemma Persello</t>
+          <t>Hanli Janse van Rensburg</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Senior Social Media Strategist</t>
+          <t>Office Administration &amp; PA</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>gemma@mag.cr</t>
+          <t>hanli@mag.cr</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1092,45 +1092,41 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.html</t>
+          <t>Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gemma_Persello.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Gemma_Persello.gif</t>
+          <t>Hanli_Janse_van_Rensburg.gif</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus Van Niekerk</t>
+          <t>Jade Weir-Smith</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>CFO - Junior Partner</t>
+          <t>Junior Growth Marketer</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>gerrie@mag.cr</t>
+          <t>jade@mag.cr</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>084 200 0823</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1140,17 +1136,17 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.html</t>
+          <t>Jade_Weir-Smith.html</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gerhardus_Van_Niekerk.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jade_Weir-Smith.html</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Gerhardus_Van_Niekerk.gif</t>
+          <t>Jade_Weir-Smith.gif</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
@@ -1163,17 +1159,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Guy Zack</t>
+          <t>Jomarie Voges</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Animation Lead</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Guy@mag.cr</t>
+          <t>jomarie@mag.cr</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1188,17 +1184,17 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.html</t>
+          <t>Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Guy_Zack.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Guy_Zack.gif</t>
+          <t>Jomarie_Voges.gif</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
@@ -1211,17 +1207,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Hanli Janse van Rensburg</t>
+          <t>Lani Bruwer</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Office Administration &amp; PA</t>
+          <t>Web Developer &amp; Information Architect</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>hanli@mag.cr</t>
+          <t>lani@mag.cr</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1236,36 +1232,40 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Hanli_Janse_van_Rensburg.html</t>
+          <t>Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Hanli_Janse_van_Rensburg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hanli_Janse_van_Rensburg.gif</t>
+          <t>Lani_Bruwer.gif</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Jade Weir-Smith</t>
+          <t>LeeAnn Visser</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Junior Growth Marketer</t>
+          <t>Video Producer</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>jade@mag.cr</t>
+          <t>lee@mag.cr</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Jade_Weir-Smith.html</t>
+          <t>LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jade_Weir-Smith.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Jade_Weir-Smith.gif</t>
+          <t>LeeAnn_Visser.gif</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Jomarie Voges</t>
+          <t>Marie Bredenkamp</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>jomarie@mag.cr</t>
+          <t>marie@mag.cr</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>076 943 5538</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1328,17 +1328,17 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.html</t>
+          <t>Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jomarie_Voges.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Jomarie_Voges.gif</t>
+          <t>Marie_Hentschel.gif</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr"/>
@@ -1351,22 +1351,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Kayla Spinelli</t>
+          <t>Marku Boshoff</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Office Administration/PA</t>
+          <t>Video Editor</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Kayla@mag.cr</t>
+          <t>marku@mag.cr</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>081 476 6721</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1376,17 +1376,17 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.html</t>
+          <t>Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kayla_Spinelli.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Kayla_Spinelli.gif</t>
+          <t>Marku_Boshoff.gif</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr"/>
@@ -1399,22 +1399,22 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Kendel Falkson</t>
+          <t>Martin Frank</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>PR Agent</t>
+          <t>Creative Director</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Kendel@mag.cr</t>
+          <t>martin@mag.cr</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>082 905 2656</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1424,17 +1424,17 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.html</t>
+          <t>Martin_Frank.html</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Kendel_Falkson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Kendel_Falkson.gif</t>
+          <t>Martin_Frank.gif</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr"/>
@@ -1447,17 +1447,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Lani Bruwer</t>
+          <t>Monique Myburgh</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Web Developer &amp; Information Architect</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>lani@mag.cr</t>
+          <t>monique@mag.cr</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1472,17 +1472,17 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.html</t>
+          <t>Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lani_Bruwer.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Lani_Bruwer.gif</t>
+          <t>Monique_Myburgh.gif</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr"/>
@@ -1495,17 +1495,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn Visser</t>
+          <t>Noël Scholtz</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Video Producer</t>
+          <t>Director of Video</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>lee@mag.cr</t>
+          <t>noel@mag.cr</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1520,17 +1520,17 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.html</t>
+          <t>Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/LeeAnn_Visser.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>LeeAnn_Visser.gif</t>
+          <t>Noel_Scholtz.gif</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
@@ -1543,22 +1543,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Marie Bredenkamp</t>
+          <t>Nuhaa Davis</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Account Director</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>marie@mag.cr</t>
+          <t>Nuhaa@mag.cr</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>076 943 5538</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1568,17 +1568,17 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.html</t>
+          <t>Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marie_Hentschel.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Marie_Hentschel.gif</t>
+          <t>Nuhaa_Davis.gif</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr"/>
@@ -1591,17 +1591,17 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Marku Boshoff</t>
+          <t>Portia Matha</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Video Editor</t>
+          <t>Junior Web Developer</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>marku@mag.cr</t>
+          <t>portia@mag.cr</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.html</t>
+          <t>Portia_Matha.html</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Marku_Boshoff.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Marku_Boshoff.gif</t>
+          <t>Portia_Matha.gif</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
@@ -1639,17 +1639,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Martin Frank</t>
+          <t>Reece Hurley</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Creative Director</t>
+          <t>Junior Designer Intern</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>martin@mag.cr</t>
+          <t>reece@mag.cr</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1664,17 +1664,17 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.html</t>
+          <t>Reece_Hurley.html</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Martin_Frank.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Martin_Frank.gif</t>
+          <t>Reece_Hurley.gif</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr"/>
@@ -1687,22 +1687,22 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Micaela Cox</t>
+          <t>Riëtte Bester</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Motion Graphics Designer</t>
+          <t>Copywriter</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Micaela@mag.cr</t>
+          <t>riette@mag.cr</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>082 977 5880</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1712,17 +1712,17 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.html</t>
+          <t>Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Micaela_Cox.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Micaela_Cox.gif</t>
+          <t>Riette_Bester.gif</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Monique Myburgh</t>
+          <t>Ruan Killian</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>monique@mag.cr</t>
+          <t>ruan@mag.cr</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1760,17 +1760,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.html</t>
+          <t>Ruan_Killian.html</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Monique_Myburgh.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Monique_Myburgh.gif</t>
+          <t>Ruan_Killian.gif</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr"/>
@@ -1783,22 +1783,22 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Nicelle Bresler</t>
+          <t>Simeon Bezuidenhout</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Senior Copywriter &amp; Strategist</t>
+          <t>Head of Video</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Nicell@mag.cr</t>
+          <t>simeon@mag.cr</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>082 295 1396</t>
+          <t>044 382 0565</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1808,17 +1808,17 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.html</t>
+          <t>Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nicelle_Bresler.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Nicelle_Bresler.gif</t>
+          <t>Simeon_Bezuidenhout.gif</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
@@ -1831,17 +1831,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Noël Scholtz</t>
+          <t>Victor Helberg</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Director of Video</t>
+          <t>Growth Marketer</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>noel@mag.cr</t>
+          <t>victor@mag.cr</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1856,17 +1856,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Noël_Scholtz.html</t>
+          <t>Victor_Helberg.html</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noël_Scholtz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Noel_Scholtz.gif</t>
+          <t>Victor_Helberg.gif</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
@@ -1879,17 +1879,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa Davis</t>
+          <t>Willem van der Merwe</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Content Creator</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa@mag.cr</t>
+          <t>Willem@mag.cr</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1904,17 +1904,17 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.html</t>
+          <t>Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Nuhaa_Davis.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Nuhaa_Davis.gif</t>
+          <t>Willem_van_der_Merwe.gif</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
@@ -1927,17 +1927,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Portia Matha</t>
+          <t>Zia Peter</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Junior Web Developer</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>portia@mag.cr</t>
+          <t>zia@mag.cr</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.html</t>
+          <t>Zia_Peter.html</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Portia_Matha.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Portia_Matha.gif</t>
+          <t>Zia_Peter.gif</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
@@ -1975,42 +1975,42 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Reece Hurley</t>
+          <t>Adrian Mass</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Junior Designer Intern</t>
+          <t>Account Manager</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>reece@mag.cr</t>
+          <t>adrian@mag.cr</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>9515519165</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.html</t>
+          <t>Adrian_Mass.html</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Reece_Hurley.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Reece_Hurley.gif</t>
+          <t>Adrian_Mass.gif</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
@@ -2023,42 +2023,42 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Riëtte Bester</t>
+          <t>Bernadette Marconi</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Senior Designer</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>riette@mag.cr</t>
+          <t>bernadette@mag.cr</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>440-523-9455</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Riëtte_Bester.html</t>
+          <t>Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Riëtte_Bester.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Riette_Bester.gif</t>
+          <t>Bernadette_Rose_Marconi.gif</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
@@ -2071,42 +2071,42 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Ruan Killian</t>
+          <t>Brad Hendrickson</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Junior Partner &amp; CCO</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>ruan@mag.cr</t>
+          <t>brad@mag.cr</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>818-231-7580</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.html</t>
+          <t>Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Ruan_Killian.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Ruan_Killian.gif</t>
+          <t>Brad_Hendrickson.gif</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr"/>
@@ -2119,42 +2119,42 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Simeon Bezuidenhout</t>
+          <t>Brett Lorenz</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Head of Video</t>
+          <t>Head of Video Production</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>simeon@mag.cr</t>
+          <t>brett@mag.cr</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>865-323-0916</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.html</t>
+          <t>Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Simeon_Bezuidenhout.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Simeon_Bezuidenhout.gif</t>
+          <t>Brett_Lorenz.gif</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr"/>
@@ -2167,42 +2167,42 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Victor Helberg</t>
+          <t>Brittany Carlson</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Growth Marketer</t>
+          <t>Account Operations Manager</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>victor@mag.cr</t>
+          <t>Brittany@mag.cr</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>951-225-5607</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.html</t>
+          <t>Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Victor_Helberg.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Victor_Helberg.gif</t>
+          <t>Brittany_Carlson.gif</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
@@ -2215,42 +2215,42 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Willem van der Merwe</t>
+          <t>Dave Korinek</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Content Creator</t>
+          <t>Founder | Chief Brand Officer</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Willem@mag.cr</t>
+          <t>dave@mag.cr</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>858-395-6726</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.html</t>
+          <t>Dave_Korinek.html</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Willem_van_der_Merwe.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Willem_van_der_Merwe.gif</t>
+          <t>Dave_Korinek.gif</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr"/>
@@ -2263,42 +2263,42 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Zia Peter</t>
+          <t>David Carrillo</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Partner &amp; ECD</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>zia@mag.cr</t>
+          <t>dc@mag.cr</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>044 382 0565</t>
+          <t>858-334-9855</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.html</t>
+          <t>David_Carrillo.html</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Zia_Peter.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Zia_Peter.gif</t>
+          <t>David_Carrillo.gif</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Adrian Mass</t>
+          <t>Eric Kroupa</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Account Manager</t>
+          <t>Director of Creative Strategy</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>adrian@mag.cr</t>
+          <t>eric@mag.cr</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>9515519165</t>
+          <t>636-236-8584</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.html</t>
+          <t>Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Adrian_Mass.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Adrian_Mass.gif</t>
+          <t>Eric_Kroupa.gif</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
@@ -2359,22 +2359,22 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Bernadette Marconi</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Senior Designer</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>bernadette@mag.cr</t>
+          <t>gabriel@mag.cr</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>440-523-9455</t>
+          <t>+49 151 26044084</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2384,17 +2384,17 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Bernadette_Rose_Marconi.html</t>
+          <t>Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Bernadette_Rose_Marconi.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Bernadette_Rose_Marconi.gif</t>
+          <t>Gabriel_Arias.gif</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
@@ -2407,22 +2407,22 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Brad Hendrickson</t>
+          <t>Jorge Ramirez</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Junior Partner &amp; CCO</t>
+          <t>Head of Web Development</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>brad@mag.cr</t>
+          <t>jorge@mag.cr</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>818-231-7580</t>
+          <t>+502 5874-8315</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2432,17 +2432,17 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.html</t>
+          <t>Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brad_Hendrickson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Brad_Hendrickson.gif</t>
+          <t>Jorge_Ramirez.gif</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr"/>
@@ -2455,22 +2455,22 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Brett Lorenz</t>
+          <t>Lauren Spinelli</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Head of Video Production</t>
+          <t>Account Director</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>brett@mag.cr</t>
+          <t>lauren@mag.cr</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>865-323-0916</t>
+          <t>951-775-2078</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2480,17 +2480,17 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.html</t>
+          <t>Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brett_Lorenz.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Brett_Lorenz.gif</t>
+          <t>Lauren_Spinelli.gif</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr"/>
@@ -2503,22 +2503,22 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Brittany Carlson</t>
+          <t>Mani Salazar</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Account Operations Manager</t>
+          <t>Design Director</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Brittany@mag.cr</t>
+          <t>mani@mag.cr</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>951-225-5607</t>
+          <t>858-610-5380</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2528,17 +2528,17 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.html</t>
+          <t>Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Brittany_Carlson.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Brittany_Carlson.gif</t>
+          <t>Manuel_Salazar.gif</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
@@ -2551,22 +2551,22 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Dave Korinek</t>
+          <t>Matt Simpson</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Founder | Chief Brand Officer</t>
+          <t>Partner &amp; COO</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>dave@mag.cr</t>
+          <t>matt@mag.cr</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>858-395-6726</t>
+          <t>858-705-2490</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2576,17 +2576,17 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.html</t>
+          <t>Matt_Simpson.html</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Dave_Korinek.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Dave_Korinek.gif</t>
+          <t>Matt_Simpson.gif</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
@@ -2599,22 +2599,22 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>David Carrillo</t>
+          <t>Mia Pitino</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Partner &amp; ECD</t>
+          <t>HR/Operations Manager</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>dc@mag.cr</t>
+          <t>mia@mag.cr</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>858-334-9855</t>
+          <t>858-395-7142</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2624,17 +2624,17 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>David_Carrillo.html</t>
+          <t>Mia_Pitino.html</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/David_Carrillo.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>David_Carrillo.gif</t>
+          <t>Mia_Pitino.gif</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr"/>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Eric Kroupa</t>
+          <t>Noah Korinek</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Director of Creative Strategy</t>
+          <t>Designer</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>eric@mag.cr</t>
+          <t>noah@mag.cr</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>636-236-8584</t>
+          <t>951-553-5340</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2672,17 +2672,17 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Eric_Kroupa.html</t>
+          <t>Noah_Korinek.html</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Eric_Kroupa.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Eric_Kroupa.gif</t>
+          <t>Noah_Korinek.gif</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
@@ -2695,22 +2695,22 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>Owen Korinek</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Web Developer</t>
+          <t>Videographer/Editor</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>gabriel@mag.cr</t>
+          <t>owen@mag.cr</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>+49 151 26044084</t>
+          <t>9515955535</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -2720,17 +2720,17 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Gabriel_Arias.html</t>
+          <t>Owen_Korinek.html</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Gabriel_Arias.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Gabriel_Arias.gif</t>
+          <t>Owen_Korinek.gif</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr"/>
@@ -2743,22 +2743,22 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Jorge Ramirez</t>
+          <t>Thomas Condry</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Head of Web Development</t>
+          <t>Senior Digital and Motion Designer</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>jorge@mag.cr</t>
+          <t>thomas@mag.cr</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>+502 5874-8315</t>
+          <t>909-210-7305</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2768,361 +2768,25 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Jorge_Ramirez.html</t>
+          <t>Thomas_Condry.html</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Jorge_Ramirez.html</t>
+          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Jorge_Ramirez.gif</t>
+          <t>Thomas_Condry.gif</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr"/>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Lauren Spinelli</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Account Director</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>lauren@mag.cr</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>951-775-2078</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Lauren_Spinelli.html</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Lauren_Spinelli.html</t>
-        </is>
-      </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>Lauren_Spinelli.gif</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>Mani Salazar</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>Design Director</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>mani@mag.cr</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>858-610-5380</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Manuel_Salazar.html</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Manuel_Salazar.html</t>
-        </is>
-      </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>Manuel_Salazar.gif</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>Matt Simpson</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>Partner &amp; COO</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>matt@mag.cr</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>858-705-2490</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>Matt_Simpson.html</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Matt_Simpson.html</t>
-        </is>
-      </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>Matt_Simpson.gif</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>Mia Pitino</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>HR/Operations Manager</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>mia@mag.cr</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>858-395-7142</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Mia_Pitino.html</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Mia_Pitino.html</t>
-        </is>
-      </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>Mia_Pitino.gif</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>Noah Korinek</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Designer</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>noah@mag.cr</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>951-553-5340</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>Noah_Korinek.html</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Noah_Korinek.html</t>
-        </is>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>Noah_Korinek.gif</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Owen Korinek</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>Videographer/Editor</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>owen@mag.cr</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>9515955535</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Owen_Korinek.html</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Owen_Korinek.html</t>
-        </is>
-      </c>
-      <c r="I54" s="3" t="inlineStr">
-        <is>
-          <t>Owen_Korinek.gif</t>
-        </is>
-      </c>
-      <c r="J54" s="5" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Keep</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>Thomas Condry</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>Senior Digital and Motion Designer</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>thomas@mag.cr</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>909-210-7305</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>Thomas_Condry.html</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>https://magn3tic.github.io/mag-signatures/pages/Thomas_Condry.html</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>Thomas_Condry.gif</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J55"/>
+  <autoFilter ref="A1:J48"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
+    <dataValidation sqref="A2:A48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Status" prompt="Leave blank or Keep to publish. Remove deletes the page on the next build." type="list">
       <formula1>"Keep,Remove"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3174,13 +2838,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3211,7 +2868,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Every person who currently has a signature page. 54 rows.</t>
+          <t>Every person who currently has a signature page. 47 rows.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New roles: Portia Matha is Web Developer, Lani Bruwer is Information Architect
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAG-signatures-master.xlsx
+++ b/MAG-signatures-master.xlsx
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Web Developer &amp; Information Architect</t>
+          <t>Information Architect</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Junior Web Developer</t>
+          <t>Web Developer</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">

</xml_diff>